<commit_message>
Tablas_Stock archivo — Abr-2026
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock_2026_04.xlsx
+++ b/Tablas/Tablas_Stock_2026_04.xlsx
@@ -29,20 +29,14 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002E4057"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -64,8 +58,8 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -458,7 +452,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>5.085 incidentes en abril (+9% vs marzo 4.690). Residuos y Limpieza concentra el 60% del volumen (3.046). Alumbrado y Transito crecen 19% y 21% respectivamente.</t>
+          <t>Total 5065 incidentes. Top areas: Residuos 3033 (60%), Alumbrado 621 (12%).</t>
         </is>
       </c>
     </row>
@@ -470,7 +464,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>76% de cierre global (+8 pp vs marzo 67.5%). Alumbrado 84% y Residuos 85% traccionan el resultado. Calles y Veredas con 7% es el caso critico del mes.</t>
+          <t>73.5% (+6.0 pp vs Mar-2026). Cumplido real 72.5%, Cancelado 1.1%.</t>
         </is>
       </c>
     </row>
@@ -482,7 +476,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>40% de cumplimiento SLA (-11 pp vs marzo 50.6%). Alumbrado lidera con 69%; Ctrl Actividades Comerciales en 4% y Espacio Publico en 19% son los mas criticos.</t>
+          <t>31.0% (-19.6 pp vs Mar-2026). Promedio 4.3 dias para incidentes cerrados.</t>
         </is>
       </c>
     </row>
@@ -494,7 +488,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>63% de satisfaccion (+2 pp vs marzo 61.4%). Tasa de respuesta 20% (encuestas sobre total incidentes). Alumbrado 79% y Transito 79% destacan positivamente.</t>
+          <t>63.2% (+1.8 pp vs Mar-2026). Tasa respuesta 16.8% (850 encuestas sobre 5065 incidentes).</t>
         </is>
       </c>
     </row>
@@ -536,7 +530,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cierre 85% sobre 621 incidentes (+10 pp vs marzo); SLA 58%. Alta gestion interna (51%). Luminarias apagadas concentran el 65% del volumen.</t>
+          <t>Cierre 85% sobre 621 incidentes; 'Luminaria superior e inferior apagada durante la noche' lidera con 402 casos (89% cierre). Gestion interna 51% del total.</t>
         </is>
       </c>
     </row>
@@ -548,7 +542,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cierre critico: 35% sobre 146 incidentes. Arboles obstruyendo señales concentran 44% del stock con solo 20% de cierre. Dias prom 7.5.</t>
+          <t>Cierre bajo 35% sobre 146 incidentes; 'Árbol obstruye semáforo/luminaria/cartel/etc.' lidera con 64 casos (20% cierre). SLA 18%, sat 25%.</t>
         </is>
       </c>
     </row>
@@ -560,7 +554,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cierre 7% sobre 282 incidentes — situacion critica. Baches y cordones con &lt;10% de resolucion. Muestra encuesta insuficiente (1.4%).</t>
+          <t>Cierre critico 7% sobre 282 incidentes; 'Bache en calle de asfalto' lidera con 104 casos (10% cierre). Sat 25% (muestra insuficiente).</t>
         </is>
       </c>
     </row>
@@ -572,7 +566,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cierre 58% sobre 89 incidentes; SLA critico 2%. Ruidos molestos y falta de habilitacion concentran el 60% del volumen.</t>
+          <t>Cierre moderado 58% sobre 89 incidentes; 'Otros ruidos molestos' lidera con 27 casos (48% cierre). SLA 2% — critico.</t>
         </is>
       </c>
     </row>
@@ -584,7 +578,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cierre 61% sobre 344 incidentes; roedores resueltos al 92% (165 casos). Cables cortados con 4% de cierre representan alerta persistente.</t>
+          <t>Cierre moderado 61% sobre 344 incidentes; 'Roedores en espacio público' lidera con 165 casos (92% cierre). SLA 12%, sat 51%.</t>
         </is>
       </c>
     </row>
@@ -596,7 +590,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cierre 82% sobre 3033 incidentes — area de mayor volumen (60% del total). SLA 28%; reciclables con solo 27% de cierre.</t>
+          <t>Cierre 82% sobre 3033 incidentes; 'Falta de barrido o barrido deficiente' lidera con 820 casos (77% cierre). SLA 28%, sat 61%.</t>
         </is>
       </c>
     </row>
@@ -608,7 +602,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cierre 71% sobre 550 incidentes. Vehiculos abandonados dominan (369 casos, 79% cierre). Vehiculos mal estacionados con 6% de cierre.</t>
+          <t>Cierre 71% sobre 550 incidentes; 'Vehículos Abandonados' lidera con 369 casos (79% cierre). Sat 83% (muestra insuficiente).</t>
         </is>
       </c>
     </row>
@@ -623,7 +617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -669,192 +663,192 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>NUEVA</t>
+          <t>PERSISTE</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Abr-2026</t>
+          <t>Feb-2026</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Alumbrado Publico</t>
+          <t>Arbolado y Plazas</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Tasa repeticion alta</t>
+          <t>Cierre bajo (area)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>91.6%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>%Rep 91.6% (umbral &gt;50%).</t>
+          <t>Tercer mes debajo de 50%: cierre 29% (-7pp), 41% Cancelado en cerrados, Sin Asignar elevado. En abril: cierre 35% — persiste debajo de 50%.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>NUEVA</t>
+          <t>PERSISTE</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Abr-2026</t>
+          <t>Feb-2026</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Arbolado y Plazas</t>
+          <t>Control de Actividades Comerciales</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo</t>
+          <t>SLA critico (area)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>34.9%</t>
+          <t>2%</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Cierre 34.9% (umbral &lt;50%). Cumplido real 30.8%.</t>
+          <t>SLA 16% — segundo mes consecutivo debajo de 30%. Dias promedio 4.4. En abril: SLA 2% — sigue por debajo del umbral.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>NUEVA</t>
+          <t>PERSISTE</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Abr-2026</t>
+          <t>Feb-2026</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Arbolado y Plazas</t>
+          <t>Control de Actividades Comerciales</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>SLA bajo</t>
+          <t>Satisfaccion baja</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>SLA 18.5% (umbral &lt;30%).</t>
+          <t>Satisfaccion 15% con 80% de encuestados insatisfechos (16/20). Cierre 81% no se traduce en percepcion de resolucion. En abril: satisfaccion 18% — persiste baja.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>NUEVA</t>
+          <t>PERSISTE</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Abr-2026</t>
+          <t>Feb-2026</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Arbolado y Plazas</t>
+          <t>Control del Espacio Publico</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Dias promedio alto</t>
+          <t>SLA bajo (area)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>7.5 dias</t>
+          <t>12%</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Promedio de resolucion 7.5 dias (umbral &gt;7).</t>
+          <t>SLA 29% — segundo mes consecutivo debajo de 30%. Poste mal estado: cierre 23% en 37 casos. En abril: SLA 12% — sigue por debajo del umbral.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>NUEVA</t>
+          <t>PERSISTE</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Abr-2026</t>
+          <t>Mar-2026</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Arbolado y Plazas</t>
+          <t>Calles y Veredas</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Tasa repeticion alta</t>
+          <t>Cierre critico (area)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>93.2%</t>
+          <t>7%</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>%Rep 93.2% (umbral &gt;50%).</t>
+          <t>Cierre colapso de 81% a 34% (-49pp). Bache asfalto 86 casos bajo cierre, Cordon 22% en 46 casos. Satisfaccion 14%. En abril: cierre 7% — persiste debajo de 50%.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>NUEVA</t>
+          <t>PERSISTE</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Abr-2026</t>
+          <t>Mar-2026</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Arbolado y Plazas</t>
+          <t>Control del Espacio Publico</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo por tipo</t>
+          <t>Poste en mal estado / sin mantenimiento</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>20.3% (64 casos)</t>
+          <t>cierre bajo</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Árbol obstruye semáforo/luminaria/cartel/etc.': cierre 20.3% con 64 casos (umbral &lt;40% para volumen &gt;20).</t>
+          <t>37 casos con 23% cierre. Poste quebrado/cortado 20% en 5 casos. En abril: tipo sigue con cierre bajo — ver hallazgos por tipo de area.</t>
         </is>
       </c>
     </row>
@@ -871,22 +865,22 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Arbolado y Plazas</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo</t>
+          <t>SLA critico (area)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Cierre 7.1% (umbral &lt;50%). Cumplido real 6.0%.</t>
+          <t>SLA 18% en abril (umbral &lt;30%). Tercer o nuevo mes en zona critica.</t>
         </is>
       </c>
     </row>
@@ -903,22 +897,22 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Arbolado y Plazas</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>SLA bajo</t>
+          <t>Dias promedio alto</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>12.4%</t>
+          <t>7.5 dias</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>SLA 12.4% (umbral &lt;30%).</t>
+          <t>Tiempo promedio de resolucion 7.5 dias en abril (umbral &gt;7).</t>
         </is>
       </c>
     </row>
@@ -935,22 +929,22 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Arbolado y Plazas</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Tasa repeticion alta</t>
+          <t>Cierre bajo — Árbol obstruye semáforo/luminaria/cartel/etc.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>79.1%</t>
+          <t>20% (64 casos)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>%Rep 79.1% (umbral &gt;50%).</t>
+          <t>Tipo 'Árbol obstruye semáforo/luminaria/cartel/etc.': cierre 20% con 64 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -972,17 +966,17 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo por tipo</t>
+          <t>Cierre bajo (area)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>9.6% (104 casos)</t>
+          <t>7%</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Bache en calle de asfalto': cierre 9.6% con 104 casos (umbral &lt;40% para volumen &gt;20).</t>
+          <t>Cierre 7% en abril (umbral &lt;50%). Cumplido real 6%.</t>
         </is>
       </c>
     </row>
@@ -1004,17 +998,17 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo por tipo</t>
+          <t>SLA critico (area)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>3.1% (65 casos)</t>
+          <t>12%</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Reparación/construcción de cordón': cierre 3.1% con 65 casos (umbral &lt;40% para volumen &gt;20).</t>
+          <t>SLA 12% en abril (umbral &lt;30%). Tercer o nuevo mes en zona critica.</t>
         </is>
       </c>
     </row>
@@ -1036,17 +1030,17 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo por tipo</t>
+          <t>Muestra encuesta insuficiente</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2.9% (34 casos)</t>
+          <t>Tasa 1.4%</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Bache en calle de hormigón': cierre 2.9% con 34 casos (umbral &lt;40% para volumen &gt;20).</t>
+          <t>Tasa de respuesta encuesta 1.4% (umbral &lt;5%). Datos de satisfaccion no representativos.</t>
         </is>
       </c>
     </row>
@@ -1068,17 +1062,17 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo por tipo</t>
+          <t>Cierre bajo — Bache en calle de asfalto</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>4.8% (21 casos)</t>
+          <t>10% (104 casos)</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Reparación de rampa de accesibilidad': cierre 4.8% con 21 casos (umbral &lt;40% para volumen &gt;20).</t>
+          <t>Tipo 'Bache en calle de asfalto': cierre 10% con 104 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1100,17 +1094,17 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Muestra encuesta insuficiente</t>
+          <t>Cierre bajo — Reparación/construcción de cordón</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Tasa 1.4%</t>
+          <t>3% (65 casos)</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Tasa de respuesta encuesta 1.4% (umbral &lt;5%). Datos de satisfaccion no representativos.</t>
+          <t>Tipo 'Reparación/construcción de cordón': cierre 3% con 65 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1127,22 +1121,22 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Control de Actividades Comerciales</t>
+          <t>Calles y Veredas</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>SLA bajo</t>
+          <t>Cierre bajo — Bache en calle de hormigón</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>2.2%</t>
+          <t>3% (34 casos)</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>SLA 2.2% (umbral &lt;30%).</t>
+          <t>Tipo 'Bache en calle de hormigón': cierre 3% con 34 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1159,22 +1153,22 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Control de Actividades Comerciales</t>
+          <t>Calles y Veredas</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Dias promedio alto</t>
+          <t>Cierre bajo — Reparación de rampa de accesibilidad</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>7.1 dias</t>
+          <t>5% (21 casos)</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Promedio de resolucion 7.1 dias (umbral &gt;7).</t>
+          <t>Tipo 'Reparación de rampa de accesibilidad': cierre 5% con 21 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1196,17 +1190,17 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Tasa repeticion alta</t>
+          <t>Dias promedio alto</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>97.8%</t>
+          <t>7.1 dias</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>%Rep 97.8% (umbral &gt;50%).</t>
+          <t>Tiempo promedio de resolucion 7.1 dias en abril (umbral &gt;7).</t>
         </is>
       </c>
     </row>
@@ -1228,17 +1222,17 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>SLA bajo</t>
+          <t>SLA critico (area)</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12%</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>SLA 12.5% (umbral &lt;30%).</t>
+          <t>SLA 12% en abril (umbral &lt;30%). Tercer o nuevo mes en zona critica.</t>
         </is>
       </c>
     </row>
@@ -1260,17 +1254,17 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Tasa repeticion alta</t>
+          <t>Cierre bajo — Cable cortado</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>86.6%</t>
+          <t>4% (55 casos)</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>%Rep 86.6% (umbral &gt;50%).</t>
+          <t>Tipo 'Cable cortado': cierre 4% con 55 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1292,17 +1286,17 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo por tipo</t>
+          <t>Cierre bajo — Poste en mal estado/sin mantenimiento</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>3.6% (55 casos)</t>
+          <t>23% (22 casos)</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Cable cortado': cierre 3.6% con 55 casos (umbral &lt;40% para volumen &gt;20).</t>
+          <t>Tipo 'Poste en mal estado/sin mantenimiento': cierre 23% con 22 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1319,22 +1313,22 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Control del Espacio Publico</t>
+          <t>Residuos y Limpieza</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo por tipo</t>
+          <t>SLA critico (area)</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>22.7% (22 casos)</t>
+          <t>28%</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Poste en mal estado/sin mantenimiento': cierre 22.7% con 22 casos (umbral &lt;40% para volumen &gt;20).</t>
+          <t>SLA 28% en abril (umbral &lt;30%). Tercer o nuevo mes en zona critica.</t>
         </is>
       </c>
     </row>
@@ -1356,17 +1350,17 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>SLA bajo</t>
+          <t>Cierre bajo — Falta de recolección de residuos reciclables (Prog</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>27.9%</t>
+          <t>27% (55 casos)</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>SLA 27.9% (umbral &lt;30%).</t>
+          <t>Tipo 'Falta de recolección de residuos reciclables (Programa Día Verde)': cierre 27% con 55 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1383,342 +1377,22 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Residuos y Limpieza</t>
+          <t>Transito</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Tasa repeticion alta</t>
+          <t>Muestra encuesta insuficiente</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>92.7%</t>
+          <t>Tasa 4.4%</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>%Rep 92.7% (umbral &gt;50%).</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Residuos y Limpieza</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>Cierre bajo por tipo</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>27.3% (55 casos)</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>Tipo 'Falta de recolección de residuos reciclables (Programa Día Verde)': cierre 27.3% con 55 casos (umbral &lt;40% para volumen &gt;20).</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Transito</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>Muestra encuesta insuficiente</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>Tasa 4.4%</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
           <t>Tasa de respuesta encuesta 4.4% (umbral &lt;5%). Datos de satisfaccion no representativos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>Proceso batch detectado</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>13 cierres/min</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>Usuario lg@mantelectric.com: 13 cierres en 1 minuto (2026-04-13 08:30:00).</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Proceso batch detectado</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>13 cierres/min</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>Usuario lg@mantelectric.com: 13 cierres en 1 minuto (2026-04-13 08:31:00).</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>Proceso batch detectado</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>15 cierres/min</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>Usuario lg@mantelectric.com: 15 cierres en 1 minuto (2026-04-14 08:32:00).</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>Proceso batch detectado</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>14 cierres/min</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>Usuario lg@mantelectric.com: 14 cierres en 1 minuto (2026-04-14 08:40:00).</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>Proceso batch detectado</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>12 cierres/min</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>Usuario lg@mantelectric.com: 12 cierres en 1 minuto (2026-04-17 08:34:00).</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Proceso batch detectado</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>17 cierres/min</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Usuario lg@mantelectric.com: 17 cierres en 1 minuto (2026-04-22 09:02:00).</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>Proceso batch detectado</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>13 cierres/min</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>Usuario lg@mantelectric.com: 13 cierres en 1 minuto (2026-04-24 08:31:00).</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>Proceso batch detectado</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>12 cierres/min</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>Usuario lg@mantelectric.com: 12 cierres en 1 minuto (2026-04-29 08:33:00).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stock_Alertas corregido — logica transicion Abr-2026
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock_2026_04.xlsx
+++ b/Tablas/Tablas_Stock_2026_04.xlsx
@@ -617,7 +617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -779,12 +779,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>19%</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>SLA 29% — segundo mes consecutivo debajo de 30%. Poste mal estado: cierre 23% en 37 casos. En abril: SLA 12% — sigue por debajo del umbral.</t>
+          <t>SLA 29% en marzo — segundo mes consecutivo debajo de 30%. En abril: SLA 19% — tercer mes en zona critica.</t>
         </is>
       </c>
     </row>
@@ -843,12 +843,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>cierre bajo</t>
+          <t>23% (22 casos)</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>37 casos con 23% cierre. Poste quebrado/cortado 20% en 5 casos. En abril: tipo sigue con cierre bajo — ver hallazgos por tipo de area.</t>
+          <t>37 casos en marzo con 23% cierre. En abril: 22 casos con 23% cierre — patron de cierre bajo sin mejora.</t>
         </is>
       </c>
     </row>
@@ -870,17 +870,17 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>SLA critico (area)</t>
+          <t>Dias promedio alto</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>8 dias</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>SLA 18% en abril (umbral &lt;30%).</t>
+          <t>Promedio de resolucion 8 dias en abril (umbral &gt;7).</t>
         </is>
       </c>
     </row>
@@ -902,17 +902,17 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Dias promedio alto</t>
+          <t>Cierre bajo — Árbol obstruye semáforo/luminaria/cartel/etc.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>7.5 dias</t>
+          <t>20% (64 casos)</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Tiempo promedio de resolucion 7.5 dias en abril (umbral &gt;7).</t>
+          <t>Tipo 'Árbol obstruye semáforo/luminaria/cartel/etc.': cierre 20% con 64 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -929,22 +929,22 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Arbolado y Plazas</t>
+          <t>Calles y Veredas</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo — Árbol obstruye semáforo/luminaria/cartel/etc.</t>
+          <t>Muestra encuesta insuficiente</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>20% (64 casos)</t>
+          <t>Tasa 1.4%</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Árbol obstruye semáforo/luminaria/cartel/etc.': cierre 20% con 64 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
+          <t>Tasa de respuesta encuesta 1.4% (umbral &lt;5%). Datos de satisfaccion no representativos.</t>
         </is>
       </c>
     </row>
@@ -966,17 +966,17 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>SLA critico (area)</t>
+          <t>Cierre bajo — Bache en calle de asfalto</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>10% (104 casos)</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>SLA 12% en abril (umbral &lt;30%).</t>
+          <t>Tipo 'Bache en calle de asfalto': cierre 10% con 104 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -998,17 +998,17 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Muestra encuesta insuficiente</t>
+          <t>Cierre bajo — Reparación/construcción de cordón</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Tasa 1.4%</t>
+          <t>3% (65 casos)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Tasa de respuesta encuesta 1.4% (umbral &lt;5%). Datos de satisfaccion no representativos.</t>
+          <t>Tipo 'Reparación/construcción de cordón': cierre 3% con 65 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1030,17 +1030,17 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo — Bache en calle de asfalto</t>
+          <t>Cierre bajo — Bache en calle de hormigón</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>10% (104 casos)</t>
+          <t>3% (34 casos)</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Bache en calle de asfalto': cierre 10% con 104 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
+          <t>Tipo 'Bache en calle de hormigón': cierre 3% con 34 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1062,17 +1062,17 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo — Reparación/construcción de cordón</t>
+          <t>Cierre bajo — Reparación de rampa de accesibilidad</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>3% (65 casos)</t>
+          <t>5% (21 casos)</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Reparación/construcción de cordón': cierre 3% con 65 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
+          <t>Tipo 'Reparación de rampa de accesibilidad': cierre 5% con 21 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1089,22 +1089,22 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Control de Actividades Comerciales</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo — Bache en calle de hormigón</t>
+          <t>Dias promedio alto</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>3% (34 casos)</t>
+          <t>7.1 dias</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Bache en calle de hormigón': cierre 3% con 34 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
+          <t>Tiempo promedio de resolucion 7.1 dias en abril (umbral &gt;7).</t>
         </is>
       </c>
     </row>
@@ -1121,22 +1121,22 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Control del Espacio Publico</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo — Reparación de rampa de accesibilidad</t>
+          <t>Cierre bajo — Cable cortado</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>5% (21 casos)</t>
+          <t>4% (55 casos)</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Reparación de rampa de accesibilidad': cierre 5% con 21 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
+          <t>Tipo 'Cable cortado': cierre 4% con 55 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1153,22 +1153,22 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Control de Actividades Comerciales</t>
+          <t>Residuos y Limpieza</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Dias promedio alto</t>
+          <t>Cierre bajo — Falta de recolección de residuos reciclables (Prog</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>7.1 dias</t>
+          <t>27% (55 casos)</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Tiempo promedio de resolucion 7.1 dias en abril (umbral &gt;7).</t>
+          <t>Tipo 'Falta de recolección de residuos reciclables (Programa Día Verde)': cierre 27% con 55 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1185,116 +1185,20 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Control del Espacio Publico</t>
+          <t>Transito</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo — Cable cortado</t>
+          <t>Muestra encuesta insuficiente</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>4% (55 casos)</t>
+          <t>Tasa 4.4%</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Tipo 'Cable cortado': cierre 4% con 55 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Residuos y Limpieza</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>SLA critico (area)</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>28%</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>SLA 28% en abril (umbral &lt;30%).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Residuos y Limpieza</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Cierre bajo — Falta de recolección de residuos reciclables (Prog</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>27% (55 casos)</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Tipo 'Falta de recolección de residuos reciclables (Programa Día Verde)': cierre 27% con 55 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Transito</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Muestra encuesta insuficiente</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Tasa 4.4%</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>Tasa de respuesta encuesta 4.4% (umbral &lt;5%). Datos de satisfaccion no representativos.</t>
         </is>

</xml_diff>

<commit_message>
fix: agrega filas RESUELTA en Stock_Alertas abril 2026
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock_2026_04.xlsx
+++ b/Tablas/Tablas_Stock_2026_04.xlsx
@@ -32,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -42,6 +42,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -62,13 +67,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -475,7 +483,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>76% (+8pp vs marzo 68%). Alumbrado 84% y Residuos 85% traccionan. Calles y Veredas cae a 7% — el mas critico del mes. Arbolado persiste en 35%.</t>
+          <t>76% (+8pp vs marzo 68%). Alumbrado 84% y Residuos 85% traccionan. Calles y Veredas cae a 7% ? el mas critico del mes. Arbolado persiste en 35%.</t>
         </is>
       </c>
     </row>
@@ -565,7 +573,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Cierre colapsa a 7% — el mas bajo del area en el periodo analizado. Volumen crece 28% con 282 casos y muestra de encuesta insuficiente (1.4%).</t>
+          <t>Cierre colapsa a 7% ? el mas bajo del area en el periodo analizado. Volumen crece 28% con 282 casos y muestra de encuesta insuficiente (1.4%).</t>
         </is>
       </c>
     </row>
@@ -628,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -674,7 +682,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>PERSISTE</t>
+          <t>RESUELTA</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -684,61 +692,61 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>ARBOLADO Y PLAZAS</t>
+          <t>TRANSITO</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Cierre bajo</t>
+          <t>Cancelado excesivo en cerrados</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>4.7%</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Cierre 29% en marzo → 35% en abril. Cuarto mes debajo de 50%. Arbol obstruye semaforo/luminaria concentra el deficit con 64 casos y 20% cierre. 11.5% de los cerrados son Cancelados.</t>
+          <t>Cancelado en cerrados baja de 39% (marzo) a 4.7% (abril). Mejora significativa. Vehiculos Abandonados deja de concentrar cancelaciones masivas.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>PERSISTE</t>
+          <t>RESUELTA</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>febrero de 2026</t>
+          <t>marzo de 2026</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>ARBOLADO Y PLAZAS</t>
+          <t>TRANSITO</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Cancelado alto en cerrados</t>
+          <t>Reparacion semaforo cierre critico</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>63%</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Cancelado sube de 41% (marzo) a 11.5% sobre total de cerrados en abril. El cierre parcial se sostiene en parte por cancelaciones.</t>
+          <t>Cierre de Reparacion de semaforo sube de 26% (marzo, 57 casos) a 63% (abril, 117 casos). Sale de zona critica con mayor volumen.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>PERSISTE</t>
+          <t>RESUELTA</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -748,29 +756,29 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>ARBOLADO Y PLAZAS</t>
+          <t>RESIDUOS Y LIMPIEZA</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Arbol obstruye cierre critico</t>
+          <t>Falta barrido variacion anomala</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>20% (64 casos)</t>
+          <t>77%</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Tipo dominante del area: 64 casos con 20% cierre en abril. En marzo: 110 casos con 14% cierre. Mejora en volumen pero el cierre sigue critico.</t>
+          <t>Cierre de Falta barrido sube de 43% (marzo) a 77% (abril). El volumen sube a 820 casos pero el cierre se normaliza. Alerta de variacion resuelta.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>PERSISTE</t>
+          <t>RESUELTA</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -780,308 +788,468 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>CALLES Y VEREDAS</t>
+          <t>RESIDUOS Y LIMPIEZA</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Cierre colapsado</t>
+          <t>Falta recoleccion organicos cierre critico</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>7%</t>
+          <t>?</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Cierre cae de 32% (marzo) a 7% (abril). Bache asfalto: 104 casos, 10% cierre. Cordon: 65 casos, 3% cierre. Hormigon: 34 casos, 3% cierre. Rampa accesibilidad: 21 casos, 5% cierre.</t>
+          <t>Sin registros de Falta recoleccion de residuos organicos/humedos en abril. En marzo: 259 casos con 11% cierre. Tipo desaparece del volumen del mes.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
+          <t>RESUELTA</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>marzo de 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Retiro restos poda arbolado variacion anomala</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Sin anomalia en abril. En marzo: 155 casos con +104% de variacion y 36% cierre. El tipo regresa a comportamiento normal en volumen y cierre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
           <t>PERSISTE</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>febrero de 2026</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Cierre bajo</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>35%</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Cierre 29% en marzo ? 35% en abril. Cuarto mes debajo de 50%. Arbol obstruye semaforo/luminaria concentra el deficit con 64 casos y 20% cierre. 11.5% de los cerrados son Cancelados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>PERSISTE</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>febrero de 2026</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Cancelado alto en cerrados</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>11.5%</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Cancelado sobre cerrados sube de 41% (marzo) a 11.5% en abril. El cierre parcial se sostiene en parte por cancelaciones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>PERSISTE</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>marzo de 2026</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Arbol obstruye cierre critico</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>20% (64 casos)</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Tipo dominante del area: 64 casos con 20% cierre en abril. En marzo: 110 casos con 14% cierre. Mejora en volumen pero el cierre sigue critico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>PERSISTE</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>marzo de 2026</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Cierre colapsado</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>7%</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Cierre cae de 32% (marzo) a 7% (abril). Bache asfalto: 104 casos, 10% cierre. Cordon: 65 casos, 3% cierre. Hormigon: 34 casos, 3% cierre. Rampa accesibilidad: 21 casos, 5% cierre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>PERSISTE</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>febrero de 2026</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>SLA critico</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>4%</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>SLA 16% en marzo → 4% en abril. Tercer mes consecutivo debajo de 30%. Dias promedio de resolucion: 9. El indicador empeora pese al volumen estable (89 casos).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>SLA 16% en marzo ? 4% en abril. Tercer mes consecutivo debajo de 30%. Dias promedio de resolucion: 9. El indicador empeora pese al volumen estable (89 casos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>PERSISTE</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>febrero de 2026</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>CONTROL DEL ESPACIO PUBLICO</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>SLA bajo</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>19%</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>SLA 29% en marzo → 19% en abril. Tercer mes debajo de 30%. Poste en mal estado (22 casos, 23% cierre) y Cable cortado (55 casos, 4% cierre) son los tipos de mayor impacto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>SLA 29% en marzo ? 19% en abril. Tercer mes debajo de 30%. Poste en mal estado (22 casos, 23% cierre) y Cable cortado (55 casos, 4% cierre) son los tipos de mayor impacto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>abril de 2026</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>CONTROL DEL ESPACIO PUBLICO</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Cable cortado cierre critico</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>4% (55 casos)</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>55 casos con solo 2 cerrados en abril (4% cierre). En marzo: 29 casos con 28% cierre. Sube el volumen y cae el cierre. Incidentes con outliers &gt;30 dias: #12329843, #12330370.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>abril de 2026</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>RESIDUOS Y LIMPIEZA</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Residuos reciclables cierre bajo</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>27% (55 casos)</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>55 casos de Residuos reciclables Dia Verde con 27% cierre en abril. Tipo con baja resolucion sostenida en el area de mayor volumen del municipio.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>abril de 2026</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>CALLES Y VEREDAS</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Muestra encuesta insuficiente</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>1.4%</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>Solo 4 respuestas de encuesta sobre 282 incidentes (1.4%). Los datos de satisfaccion (25%) no son representativos. Segundo mes con muestra reducida en el area.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>abril de 2026</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>TRANSITO</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Muestra encuesta insuficiente</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>4.4%</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>24 respuestas sobre 551 incidentes (4.4%). Satisfaccion 79% no es representativa. Persistente problema de envio de encuestas en Vehiculos Abandonados.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>abril de 2026</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Satisfaccion baja</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>18%</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Satisfaccion 18% con cierre 58%. Brecha de 40pp entre cierre y satisfaccion sugiere que los cierres no se perciben como resolucion efectiva. 12.4% tasa de respuesta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Satisfaccion 18% con cierre 58%. Brecha de 40pp entre cierre y satisfaccion: los cierres no se perciben como resolucion efectiva. 12.4% tasa de respuesta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>abril de 2026</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Dias promedio alto</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>9 dias</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>Dias promedio de resolucion: 9 dias en abril (era 6 en marzo). El incremento se da con volumen estable (-1%), lo que indica enlentecimiento operativo.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>abril de 2026</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>ARBOLADO Y PLAZAS</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>Dias promedio alto</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>8 dias</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>Dias promedio de resolucion: 8 dias en abril. Coincide con bajo cierre (35%) y alta concentracion de casos abiertos de Arbol obstruye sin resolver.</t>
         </is>

</xml_diff>

<commit_message>
fix: corregir valores del tablero y agregar alerta Transito vehiculo mal estacionado
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock_2026_04.xlsx
+++ b/Tablas/Tablas_Stock_2026_04.xlsx
@@ -28,8 +28,10 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
@@ -41,7 +43,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
+        <fgColor rgb="005B2C8D"/>
       </patternFill>
     </fill>
     <fill>
@@ -69,15 +71,17 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -448,10 +452,10 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>KPI</t>
@@ -463,44 +467,44 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="45" customHeight="1">
+      <c r="A2" t="inlineStr">
         <is>
           <t>CANTIDAD</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>5.085 incidentes en abril (+9% vs marzo 4.675). Residuos lidera con 3.046 casos. Alumbrado +19%, Transito +21%, Calles +28%. Arbolado baja -30%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+          <t>5.077 incidentes en abril (+8% vs marzo 4.675). Residuos lidera con 3.039 casos. Alumbrado +19%, Transito +21%, Calles +28%. Arbolado baja -33%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
+      <c r="A3" t="inlineStr">
         <is>
           <t>CIERRE</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>76% (+8pp vs marzo 68%). Alumbrado 84% y Residuos 85% traccionan. Calles y Veredas cae a 7% ? el mas critico del mes. Arbolado persiste en 35%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+          <t>74% (+6pp vs marzo 68%). Alumbrado 84% y Residuos 82% traccionan. Calles y Veredas cae a 7% — el mas critico del mes. Arbolado persiste en 35%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="45" customHeight="1">
+      <c r="A4" t="inlineStr">
         <is>
           <t>SLA</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>40% (-10pp vs marzo 50%). Alumbrado lidera con 69%. Ctrl Comerciales 4% y Ctrl Espacio Publico 19% concentran el deficit. Transito sube a 63%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+          <t>41% (-9pp vs marzo 50%). Alumbrado lidera con 69%. Ctrl Comerciales 4% y Ctrl Espacio Publico 19% concentran el deficit. Transito sube a 63%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="45" customHeight="1">
+      <c r="A5" t="inlineStr">
         <is>
           <t>SATISFACCION</t>
         </is>
@@ -525,11 +529,11 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Area</t>
@@ -541,8 +545,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" t="inlineStr">
         <is>
           <t>ALUMBRADO PUBLICO</t>
         </is>
@@ -553,8 +557,8 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="3" ht="40" customHeight="1">
+      <c r="A3" t="inlineStr">
         <is>
           <t>ARBOLADO Y PLAZAS</t>
         </is>
@@ -565,20 +569,20 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" t="inlineStr">
         <is>
           <t>CALLES Y VEREDAS</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Cierre colapsa a 7% ? el mas bajo del area en el periodo analizado. Volumen crece 28% con 282 casos y muestra de encuesta insuficiente (1.4%).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+          <t>Cierre colapsa a 7%, el mas bajo del area en el periodo analizado. Volumen crece 28% con 282 casos y muestra de encuesta insuficiente (1.4%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" t="inlineStr">
         <is>
           <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
         </is>
@@ -589,8 +593,8 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" t="inlineStr">
         <is>
           <t>CONTROL DEL ESPACIO PUBLICO</t>
         </is>
@@ -601,20 +605,20 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" t="inlineStr">
         <is>
           <t>RESIDUOS Y LIMPIEZA</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Cierre 85%, el mejor del municipio. Falta barrido resuelve (77%). Residuos reciclables Dia Verde con 27% cierre en 55 casos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+          <t>Cierre 82% — mejor del municipio. Falta barrido resuelve (77%). Residuos reciclables Dia Verde con 27% cierre en 55 casos es la nueva alerta del area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" t="inlineStr">
         <is>
           <t>TRANSITO</t>
         </is>
@@ -641,13 +645,13 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="80" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Estado</t>
@@ -679,7 +683,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="55" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>RESUELTA</t>
@@ -707,11 +711,11 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Cancelado en cerrados baja de 39% (marzo) a 4.7% (abril). Mejora significativa. Vehiculos Abandonados deja de concentrar cancelaciones masivas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+          <t>En febrero el 39% de los cerrados de Transito eran cancelados — anomalia persistente. En abril el porcentaje cae a 4.7%, dentro del rango operativo normal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="55" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>RESUELTA</t>
@@ -739,11 +743,11 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Cierre de Reparacion de semaforo sube de 26% (marzo, 57 casos) a 63% (abril, 117 casos). Sale de zona critica con mayor volumen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
+          <t>Reparacion de semaforo tenia 26% de cierre en marzo (117 casos pendientes). En abril sube a 63% — mejora de 37pp, sale de zona critica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="55" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>RESUELTA</t>
@@ -771,11 +775,11 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Cierre de Falta barrido sube de 43% (marzo) a 77% (abril). El volumen sube a 820 casos pero el cierre se normaliza. Alerta de variacion resuelta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+          <t>En marzo Falta barrido registro variacion anomala de volumen. En abril el cierre sube de 43% a 77% y el volumen se normaliza — alerta superada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="55" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>RESUELTA</t>
@@ -798,16 +802,16 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>sin registros</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Sin registros de Falta recoleccion de residuos organicos/humedos en abril. En marzo: 259 casos con 11% cierre. Tipo desaparece del volumen del mes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
+          <t>Falta de recoleccion de residuos organicos concentraba casos con bajo cierre en marzo. En abril no se registran casos del tipo — alerta resuelta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="55" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>RESUELTA</t>
@@ -830,16 +834,16 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>sin registros</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Sin anomalia en abril. En marzo: 155 casos con +104% de variacion y 36% cierre. El tipo regresa a comportamiento normal en volumen y cierre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
+          <t>Retiro de restos de poda/arbolado presento variacion anomala en marzo. En abril no se registran casos del tipo — alerta resuelta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="55" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>PERSISTE</t>
@@ -867,11 +871,11 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Cierre 29% en marzo ? 35% en abril. Cuarto mes debajo de 50%. Arbol obstruye semaforo/luminaria concentra el deficit con 64 casos y 20% cierre. 11.5% de los cerrados son Cancelados.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
+          <t>Arbolado y Plazas mantiene 35% de cierre en abril — tercer mes consecutivo en zona critica. Arbol obstruye semaforo/luminaria (64 casos, 20% cierre) y alta proporcion de cancelados (11.5%) concentran el problema.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="55" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>PERSISTE</t>
@@ -899,11 +903,11 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Cancelado sobre cerrados sube de 41% (marzo) a 11.5% en abril. El cierre parcial se sostiene en parte por cancelaciones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
+          <t>El 11.5% de los cierres del area son cancelaciones, por encima del 10% de referencia. Persiste desde febrero sin mejora.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="55" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>PERSISTE</t>
@@ -931,11 +935,11 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Tipo dominante del area: 64 casos con 20% cierre en abril. En marzo: 110 casos con 14% cierre. Mejora en volumen pero el cierre sigue critico.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
+          <t>Arbol obstruye semaforo/luminaria/cartel mantiene 20% de cierre con 64 casos en abril. Sin variacion respecto a marzo — el tipo concentra el deficit de cierre del area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="55" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>PERSISTE</t>
@@ -963,11 +967,11 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Cierre cae de 32% (marzo) a 7% (abril). Bache asfalto: 104 casos, 10% cierre. Cordon: 65 casos, 3% cierre. Hormigon: 34 casos, 3% cierre. Rampa accesibilidad: 21 casos, 5% cierre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
+          <t>Calles y Veredas cae de 32% en marzo a 7% en abril — 282 casos con Bache asfalto (104, 10% cierre), Cordon (65, 3% cierre) y Bache hormigon (34, 3% cierre) sin resolucion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="55" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>PERSISTE</t>
@@ -995,11 +999,11 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>SLA 16% en marzo ? 4% en abril. Tercer mes consecutivo debajo de 30%. Dias promedio de resolucion: 9. El indicador empeora pese al volumen estable (89 casos).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
+          <t>SLA de 4% por tercer mes consecutivo — el indicador mas bajo del municipio. Los tiempos de resolucion estan fuera del parametro en la totalidad del area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="55" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>PERSISTE</t>
@@ -1027,11 +1031,11 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>SLA 29% en marzo ? 19% en abril. Tercer mes debajo de 30%. Poste en mal estado (22 casos, 23% cierre) y Cable cortado (55 casos, 4% cierre) son los tipos de mayor impacto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
+          <t>SLA del area persiste en 19% en abril, sin variacion respecto a febrero-marzo. Cable cortado (55 casos, 4% cierre) y Poste en mal estado (22 casos, 23% cierre) contribuyen al indicador bajo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="55" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
@@ -1059,11 +1063,11 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>55 casos con solo 2 cerrados en abril (4% cierre). En marzo: 29 casos con 28% cierre. Sube el volumen y cae el cierre. Incidentes con outliers &gt;30 dias: #12329843, #12330370.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
+          <t>Cable cortado suma 55 casos en abril con 4% de cierre — acumulacion de casos sin resolucion. El tipo no contaba con alerta previa; en abril supera el umbral de volumen con cierre critico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="55" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
@@ -1091,11 +1095,11 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>55 casos de Residuos reciclables Dia Verde con 27% cierre en abril. Tipo con baja resolucion sostenida en el area de mayor volumen del municipio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
+          <t>Residuos reciclables Dia Verde registra 27% de cierre con 55 casos en abril. Primer mes con volumen significativo y cierre por debajo de 40%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="55" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
@@ -1123,11 +1127,11 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Solo 4 respuestas de encuesta sobre 282 incidentes (1.4%). Los datos de satisfaccion (25%) no son representativos. Segundo mes con muestra reducida en el area.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
+          <t>Tasa de respuesta de encuesta en Calles y Veredas es 1.4% (4 respuestas sobre 282 incidentes) — muestra no representativa. No es posible evaluar satisfaccion del area este mes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="55" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
@@ -1155,11 +1159,11 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>24 respuestas sobre 551 incidentes (4.4%). Satisfaccion 79% no es representativa. Persistente problema de envio de encuestas en Vehiculos Abandonados.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
+          <t>Tasa de respuesta de encuesta en Transito es 4.4% (24 respuestas sobre 551 incidentes) — por debajo del minimo para representatividad. Satisfaccion reportada (79%) no es estadisticamente confiable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="55" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
@@ -1187,11 +1191,11 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Satisfaccion 18% con cierre 58%. Brecha de 40pp entre cierre y satisfaccion: los cierres no se perciben como resolucion efectiva. 12.4% tasa de respuesta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
+          <t>Satisfaccion de 18% en Control de Actividades Comerciales con 12.4% de tasa de respuesta — el peor indicador del municipio. Ruidos molestos y falta de notificacion de resolucion concentran los comentarios negativos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="55" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
@@ -1219,11 +1223,11 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Dias promedio de resolucion: 9 dias en abril (era 6 en marzo). El incremento se da con volumen estable (-1%), lo que indica enlentecimiento operativo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
+          <t>Dias promedio de resolucion sube a 9 dias en abril — el mayor registrado para el area. Combinado con SLA 4% y satisfaccion 18%, configura la situacion mas critica del municipio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="55" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
@@ -1251,7 +1255,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Dias promedio de resolucion: 8 dias en abril. Coincide con bajo cierre (35%) y alta concentracion de casos abiertos de Arbol obstruye sin resolver.</t>
+          <t>Dias promedio de resolucion de 8 dias en Arbolado y Plazas — por encima del umbral. Se suma al cierre bajo (35%) y al alto porcentaje de cancelados (11.5%).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tablas_Stock archivo v2 - Abr-2026
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock_2026_04.xlsx
+++ b/Tablas/Tablas_Stock_2026_04.xlsx
@@ -623,7 +623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -977,12 +977,12 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>2%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>SLA 2% en abril, persiste debajo del umbral 30%.</t>
+          <t>SLA 4% en abril (tablero), persiste debajo del umbral 30%.</t>
         </is>
       </c>
     </row>
@@ -1009,12 +1009,12 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>19%</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>SLA 12% en abril, persiste debajo del umbral 30%.</t>
+          <t>SLA 19% en abril (tablero), persiste debajo del umbral 30%.</t>
         </is>
       </c>
     </row>
@@ -1036,17 +1036,17 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>SLA critico (area)</t>
+          <t>Dias promedio alto</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>8 dias</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>SLA del area 18% en abril (umbral &lt;30%). Tiempos de resolucion fuera de parametro.</t>
+          <t>Tiempo promedio de resolucion 8 dias en abril (tablero, umbral &gt;7).</t>
         </is>
       </c>
     </row>
@@ -1063,22 +1063,22 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Arbolado y Plazas</t>
+          <t>Calles y Veredas</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Dias promedio alto</t>
+          <t>Muestra encuesta insuficiente</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>7.5 dias</t>
+          <t>Tasa 1.4%</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Tiempo promedio de resolucion 7.5 dias en abril (umbral &gt;7).</t>
+          <t>Tasa de respuesta encuesta 1.4% (4 respuestas sobre 282 incidentes). Datos de satisfaccion no representativos.</t>
         </is>
       </c>
     </row>
@@ -1095,7 +1095,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Control de Actividades Comerciales</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1105,12 +1105,12 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>SLA del area 12% en abril (umbral &lt;30%). Tiempos de resolucion fuera de parametro.</t>
+          <t>SLA del area 4% en abril (tablero, umbral &lt;30%). Tiempos de resolucion fuera de parametro.</t>
         </is>
       </c>
     </row>
@@ -1127,22 +1127,22 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Control de Actividades Comerciales</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Muestra encuesta insuficiente</t>
+          <t>Dias promedio alto</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Tasa 1.4%</t>
+          <t>9 dias</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Tasa de respuesta encuesta 1.4% (4 respuestas sobre 282 incidentes). Datos de satisfaccion no representativos.</t>
+          <t>Tiempo promedio de resolucion 9 dias en abril (tablero, umbral &gt;7).</t>
         </is>
       </c>
     </row>
@@ -1159,22 +1159,22 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Control de Actividades Comerciales</t>
+          <t>Control del Espacio Publico</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>SLA critico (area)</t>
+          <t>Cierre bajo - Cable cortado</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>2%</t>
+          <t>4% (55 casos)</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>SLA del area 2% en abril (umbral &lt;30%). Tiempos de resolucion fuera de parametro.</t>
+          <t>Tipo 'Cable cortado': 55 casos en abril con 4% de cierre (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1191,22 +1191,22 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Control de Actividades Comerciales</t>
+          <t>Residuos y Limpieza</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Dias promedio alto</t>
+          <t>Cierre bajo - Falta de recolección de residuos reciclables (Pr</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>7.1 dias</t>
+          <t>27% (55 casos)</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Tiempo promedio de resolucion 7.1 dias en abril (umbral &gt;7).</t>
+          <t>Tipo 'Falta de recolección de residuos reciclables (Programa Día Verde)': 55 casos en abril con 27% de cierre (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1223,116 +1223,20 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Control del Espacio Publico</t>
+          <t>Transito</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Cierre bajo - Cable cortado</t>
+          <t>Muestra encuesta insuficiente</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>4% (55 casos)</t>
+          <t>Tasa 4.4%</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Tipo 'Cable cortado': 55 casos en abril con 4% de cierre (umbral &lt;40% con volumen &gt;=20).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Residuos y Limpieza</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>SLA critico (area)</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>28%</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>SLA del area 28% en abril (umbral &lt;30%). Tiempos de resolucion fuera de parametro.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Residuos y Limpieza</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>Cierre bajo - Falta de recolección de residuos reciclables (Pr</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>27% (55 casos)</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>Tipo 'Falta de recolección de residuos reciclables (Programa Día Verde)': 55 casos en abril con 27% de cierre (umbral &lt;40% con volumen &gt;=20).</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Transito</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>Muestra encuesta insuficiente</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>Tasa 4.4%</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>Tasa de respuesta encuesta 4.4% (24 respuestas sobre 550 incidentes). Datos de satisfaccion no representativos.</t>
         </is>

</xml_diff>